<commit_message>
refactor: rename algorithms folder to algorithms_py
</commit_message>
<xml_diff>
--- a/map.xlsx
+++ b/map.xlsx
@@ -736,7 +736,7 @@
     <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
     <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="3">
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
       <fill>
@@ -749,6 +749,13 @@
       <fill>
         <patternFill patternType="solid">
           <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="0" tint="-0.05"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1015,12 +1022,10 @@
   <dimension ref="A1:AF32"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="3.66666666666667" customWidth="1"/>
-    <col min="2" max="10" width="2.66666666666667" customWidth="1"/>
-    <col min="11" max="32" width="3.66666666666667" customWidth="1"/>
+    <col min="1" max="32" width="3.77777777777778" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32">
+    <row r="1" ht="20.4" customHeight="1" spans="1:32">
       <c r="A1" s="1"/>
       <c r="B1" s="2">
         <v>0</v>
@@ -1114,7 +1119,7 @@
       </c>
       <c r="AF1" s="1"/>
     </row>
-    <row r="2" spans="1:32">
+    <row r="2" ht="20.4" customHeight="1" spans="1:32">
       <c r="A2" s="2">
         <v>0</v>
       </c>
@@ -1212,7 +1217,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:32">
+    <row r="3" ht="20.4" customHeight="1" spans="1:32">
       <c r="A3" s="2">
         <v>1</v>
       </c>
@@ -1310,7 +1315,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:32">
+    <row r="4" ht="20.4" customHeight="1" spans="1:32">
       <c r="A4" s="2">
         <v>2</v>
       </c>
@@ -1408,7 +1413,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:32">
+    <row r="5" ht="20.4" customHeight="1" spans="1:32">
       <c r="A5" s="2">
         <v>3</v>
       </c>
@@ -1506,7 +1511,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:32">
+    <row r="6" ht="20.4" customHeight="1" spans="1:32">
       <c r="A6" s="2">
         <v>4</v>
       </c>
@@ -1604,7 +1609,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:32">
+    <row r="7" ht="20.4" customHeight="1" spans="1:32">
       <c r="A7" s="2">
         <v>5</v>
       </c>
@@ -1702,7 +1707,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:32">
+    <row r="8" ht="20.4" customHeight="1" spans="1:32">
       <c r="A8" s="2">
         <v>6</v>
       </c>
@@ -1800,7 +1805,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:32">
+    <row r="9" ht="20.4" customHeight="1" spans="1:32">
       <c r="A9" s="2">
         <v>7</v>
       </c>
@@ -1898,7 +1903,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:32">
+    <row r="10" ht="20.4" customHeight="1" spans="1:32">
       <c r="A10" s="2">
         <v>8</v>
       </c>
@@ -1996,7 +2001,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:32">
+    <row r="11" ht="20.4" customHeight="1" spans="1:32">
       <c r="A11" s="2">
         <v>9</v>
       </c>
@@ -2094,7 +2099,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:32">
+    <row r="12" ht="20.4" customHeight="1" spans="1:32">
       <c r="A12" s="2">
         <v>10</v>
       </c>
@@ -2192,7 +2197,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:32">
+    <row r="13" ht="20.4" customHeight="1" spans="1:32">
       <c r="A13" s="2">
         <v>11</v>
       </c>
@@ -2290,7 +2295,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:32">
+    <row r="14" ht="20.4" customHeight="1" spans="1:32">
       <c r="A14" s="2">
         <v>12</v>
       </c>
@@ -2388,7 +2393,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:32">
+    <row r="15" ht="20.4" customHeight="1" spans="1:32">
       <c r="A15" s="2">
         <v>13</v>
       </c>
@@ -2486,7 +2491,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:32">
+    <row r="16" ht="20.4" customHeight="1" spans="1:32">
       <c r="A16" s="2">
         <v>14</v>
       </c>
@@ -2584,7 +2589,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:32">
+    <row r="17" ht="20.4" customHeight="1" spans="1:32">
       <c r="A17" s="2">
         <v>15</v>
       </c>
@@ -2682,7 +2687,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:32">
+    <row r="18" ht="20.4" customHeight="1" spans="1:32">
       <c r="A18" s="2">
         <v>16</v>
       </c>
@@ -2780,7 +2785,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:32">
+    <row r="19" ht="20.4" customHeight="1" spans="1:32">
       <c r="A19" s="2">
         <v>17</v>
       </c>
@@ -2878,7 +2883,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:32">
+    <row r="20" ht="20.4" customHeight="1" spans="1:32">
       <c r="A20" s="2">
         <v>18</v>
       </c>
@@ -2976,7 +2981,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="1:32">
+    <row r="21" ht="20.4" customHeight="1" spans="1:32">
       <c r="A21" s="2">
         <v>19</v>
       </c>
@@ -3074,7 +3079,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:32">
+    <row r="22" ht="20.4" customHeight="1" spans="1:32">
       <c r="A22" s="2">
         <v>20</v>
       </c>
@@ -3172,7 +3177,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="1:32">
+    <row r="23" ht="20.4" customHeight="1" spans="1:32">
       <c r="A23" s="2">
         <v>21</v>
       </c>
@@ -3270,7 +3275,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="1:32">
+    <row r="24" ht="20.4" customHeight="1" spans="1:32">
       <c r="A24" s="2">
         <v>22</v>
       </c>
@@ -3368,7 +3373,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="25" spans="1:32">
+    <row r="25" ht="20.4" customHeight="1" spans="1:32">
       <c r="A25" s="2">
         <v>23</v>
       </c>
@@ -3466,7 +3471,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="1:32">
+    <row r="26" ht="20.4" customHeight="1" spans="1:32">
       <c r="A26" s="2">
         <v>24</v>
       </c>
@@ -3564,7 +3569,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="27" spans="1:32">
+    <row r="27" ht="20.4" customHeight="1" spans="1:32">
       <c r="A27" s="2">
         <v>25</v>
       </c>
@@ -3662,7 +3667,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="1:32">
+    <row r="28" ht="20.4" customHeight="1" spans="1:32">
       <c r="A28" s="2">
         <v>26</v>
       </c>
@@ -3760,7 +3765,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="29" spans="1:32">
+    <row r="29" ht="20.4" customHeight="1" spans="1:32">
       <c r="A29" s="2">
         <v>27</v>
       </c>
@@ -3858,7 +3863,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="30" spans="1:32">
+    <row r="30" ht="20.4" customHeight="1" spans="1:32">
       <c r="A30" s="2">
         <v>28</v>
       </c>
@@ -3956,7 +3961,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="31" spans="1:32">
+    <row r="31" ht="20.4" customHeight="1" spans="1:32">
       <c r="A31" s="2">
         <v>29</v>
       </c>
@@ -4054,7 +4059,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="32" spans="1:32">
+    <row r="32" ht="20.4" customHeight="1" spans="1:32">
       <c r="A32" s="1"/>
       <c r="B32" s="2">
         <v>0</v>
@@ -4150,18 +4155,18 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F25">
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2:AE24 B25:E25 G25:AE25 B26:AE31">
-    <cfRule type="cellIs" dxfId="1" priority="5" operator="equal">
+  <conditionalFormatting sqref="B2:AE31">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="7" operator="equal">
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>